<commit_message>
Iniated Verification Plan for the proc module (top module)
</commit_message>
<xml_diff>
--- a/TestPlanLAB3.xlsx
+++ b/TestPlanLAB3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lab3-Processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9DBB96-BA15-4527-89E1-59C542718F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E932D89-33FF-4B13-BA33-6D3EEEBBAF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7EA4F4C7-C520-464C-9DC5-C7C61FA541CF}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Expected Outcome</t>
   </si>
@@ -156,6 +156,18 @@
   </si>
   <si>
     <t>הזנת הערך מינוס 256 (000_000_100) ל-R1, והערך 1 ל-R2 בעזרת פקודות mvi. לאחר מכן, הזנת פקודת sub R1, R2 (010_001_010) והרצת 4 מחזורי שעון.</t>
+  </si>
+  <si>
+    <t>הזנת פקודה לא חוקית 111_111_111</t>
+  </si>
+  <si>
+    <t>לבדוק מצב defult, כלום לא משתנה</t>
+  </si>
+  <si>
+    <t>בלחיצה על הכפתור לא נקבל פידבק מהכרטיס וכל הלדים יהיו כבויים</t>
+  </si>
+  <si>
+    <t>איפוס המערכת בזמן העבודה</t>
   </si>
 </sst>
 </file>
@@ -192,7 +204,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -276,20 +288,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -309,18 +312,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="14">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -340,9 +352,7 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -350,9 +360,6 @@
           <color indexed="64"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -373,7 +380,9 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -606,8 +615,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A0F2C21D-7BA7-4ADF-9596-E9A6B7D91F6E}" name="Table1" displayName="Table1" ref="B2:F13" headerRowDxfId="13" dataDxfId="11" totalsRowDxfId="9" headerRowBorderDxfId="12" tableBorderDxfId="10">
-  <autoFilter ref="B2:F13" xr:uid="{A0F2C21D-7BA7-4ADF-9596-E9A6B7D91F6E}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A0F2C21D-7BA7-4ADF-9596-E9A6B7D91F6E}" name="Table1" displayName="Table1" ref="B2:F15" headerRowDxfId="13" dataDxfId="11" totalsRowDxfId="9" headerRowBorderDxfId="12" tableBorderDxfId="10">
+  <autoFilter ref="B2:F15" xr:uid="{A0F2C21D-7BA7-4ADF-9596-E9A6B7D91F6E}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -618,8 +627,8 @@
     <tableColumn id="1" xr3:uid="{A1C99761-FA5D-4CAC-BCF0-1D3837251535}" name="Expected Outcome" totalsRowLabel="Total" dataDxfId="8" totalsRowDxfId="7"/>
     <tableColumn id="2" xr3:uid="{5945003B-CFBB-431E-A00A-29075B00BABC}" name="Target" dataDxfId="6" totalsRowDxfId="5"/>
     <tableColumn id="3" xr3:uid="{DF17EA11-4E32-4641-91F8-86C16FA23B95}" name="Test Procedure" dataDxfId="4" totalsRowDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{5A51C804-5835-4668-98FD-4E975BF8CD31}" name="ID" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{060C108B-E6C2-46AB-9183-21514436D536}" name="Module" totalsRowFunction="count" dataDxfId="2" totalsRowDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{5A51C804-5835-4668-98FD-4E975BF8CD31}" name="ID" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{060C108B-E6C2-46AB-9183-21514436D536}" name="Module" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -942,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE16AEC-FEEA-4053-B9DA-1119D8D98FA8}">
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:F31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="46" customWidth="1"/>
@@ -1116,7 +1125,7 @@
       <c r="D12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <v>1.1000000000000001</v>
       </c>
       <c r="F12" s="6"/>
@@ -1136,18 +1145,138 @@
       </c>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
+    <row r="14" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="10"/>
+      <c r="F30" s="10"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="F31" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>